<commit_message>
feat: add 睿修 to Technical DCC leadership (翊庭、睿修) and update company logo & DMS url
</commit_message>
<xml_diff>
--- a/盛欣_盛碁網絡_營運協同與治理標準化總綱_DMS.xlsx
+++ b/盛欣_盛碁網絡_營運協同與治理標準化總綱_DMS.xlsx
@@ -684,17 +684,17 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>適用對象</t>
+          <t>文檔中心系統</t>
         </is>
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>全體營運與職能團隊 (管理、客服、財務、技術、美術、MIS)</t>
+          <t>http://10.0.0.24:8091</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>線上站點</t>
+          <t>線上戰情站點</t>
         </is>
       </c>
       <c r="F3" s="3" t="inlineStr">
@@ -785,7 +785,7 @@
       </c>
       <c r="B8" s="7" t="inlineStr">
         <is>
-          <t>翊庭</t>
+          <t>翊庭 / 睿修</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
@@ -1404,7 +1404,7 @@
       <c r="F5" s="13" t="inlineStr">
         <is>
           <t>執行部門經辦維護
-技術文管（翊庭）與主管核准</t>
+技術文管（翊庭 / 睿修）與主管核准</t>
         </is>
       </c>
       <c r="G5" s="3" t="inlineStr">
@@ -1657,7 +1657,7 @@
       </c>
       <c r="F15" s="14" t="inlineStr">
         <is>
-          <t>技術 翊庭 / 人事 芮郗</t>
+          <t>技術 翊庭 / 睿修 / 人事 芮郗</t>
         </is>
       </c>
     </row>
@@ -1689,7 +1689,7 @@
       </c>
       <c r="F16" s="13" t="inlineStr">
         <is>
-          <t>財務 玉霜 / 技術 翊庭</t>
+          <t>財務 玉霜 / 技術 翊庭 / 睿修</t>
         </is>
       </c>
     </row>
@@ -1817,7 +1817,7 @@
       </c>
       <c r="F20" s="13" t="inlineStr">
         <is>
-          <t>技術 翊庭 / MIS</t>
+          <t>技術 翊庭 / 睿修 / MIS</t>
         </is>
       </c>
     </row>
@@ -1986,7 +1986,7 @@
       </c>
       <c r="F6" s="13" t="inlineStr">
         <is>
-          <t>技術 翊庭 / 人事 芮郗</t>
+          <t>技術 翊庭 / 睿修 / 人事 芮郗</t>
         </is>
       </c>
     </row>
@@ -2018,7 +2018,7 @@
       </c>
       <c r="F7" s="14" t="inlineStr">
         <is>
-          <t>技術 翊庭</t>
+          <t>技術 翊庭 / 睿修</t>
         </is>
       </c>
     </row>
@@ -2114,7 +2114,7 @@
       </c>
       <c r="F10" s="13" t="inlineStr">
         <is>
-          <t>技術 翊庭</t>
+          <t>技術 翊庭 / 睿修</t>
         </is>
       </c>
     </row>
@@ -2146,7 +2146,7 @@
       </c>
       <c r="F11" s="14" t="inlineStr">
         <is>
-          <t>技術 翊庭</t>
+          <t>技術 翊庭 / 睿修</t>
         </is>
       </c>
     </row>
@@ -2242,7 +2242,7 @@
       </c>
       <c r="F14" s="13" t="inlineStr">
         <is>
-          <t>技術 翊庭 / 人事 芮郗</t>
+          <t>技術 翊庭 / 睿修 / 人事 芮郗</t>
         </is>
       </c>
     </row>
@@ -3164,7 +3164,7 @@
     <col width="55" customWidth="1" min="3" max="3"/>
     <col width="52" customWidth="1" min="4" max="4"/>
     <col width="21" customWidth="1" min="5" max="5"/>
-    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="25" customWidth="1" min="6" max="6"/>
     <col width="23" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
@@ -3761,7 +3761,7 @@
       </c>
       <c r="F19" s="14" t="inlineStr">
         <is>
-          <t>技術 翊庭</t>
+          <t>技術 翊庭 / 睿修</t>
         </is>
       </c>
     </row>
@@ -3825,7 +3825,7 @@
       </c>
       <c r="F21" s="14" t="inlineStr">
         <is>
-          <t>技術 翊庭 / MIS</t>
+          <t>技術 翊庭 / 睿修 / MIS</t>
         </is>
       </c>
     </row>
@@ -3857,7 +3857,7 @@
       </c>
       <c r="F22" s="13" t="inlineStr">
         <is>
-          <t>技術 翊庭</t>
+          <t>技術 翊庭 / 睿修</t>
         </is>
       </c>
     </row>
@@ -3889,7 +3889,7 @@
       </c>
       <c r="F23" s="14" t="inlineStr">
         <is>
-          <t>技術 翊庭 / MIS</t>
+          <t>技術 翊庭 / 睿修 / MIS</t>
         </is>
       </c>
     </row>
@@ -3916,7 +3916,7 @@
     <col width="55" customWidth="1" min="3" max="3"/>
     <col width="55" customWidth="1" min="4" max="4"/>
     <col width="55" customWidth="1" min="5" max="5"/>
-    <col width="24" customWidth="1" min="6" max="6"/>
+    <col width="31" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1" ht="40" customHeight="1">
@@ -4060,7 +4060,7 @@
       </c>
       <c r="F6" s="13" t="inlineStr">
         <is>
-          <t>技術 翊庭 / MIS</t>
+          <t>技術 翊庭 / 睿修 / MIS</t>
         </is>
       </c>
     </row>
@@ -4226,7 +4226,7 @@
       </c>
       <c r="E13" s="14" t="inlineStr">
         <is>
-          <t>技術 翊庭</t>
+          <t>技術 翊庭 / 睿修</t>
         </is>
       </c>
       <c r="F13" s="14" t="inlineStr">
@@ -4258,7 +4258,7 @@
       </c>
       <c r="E14" s="13" t="inlineStr">
         <is>
-          <t>技術 翊庭</t>
+          <t>技術 翊庭 / 睿修</t>
         </is>
       </c>
       <c r="F14" s="13" t="inlineStr">
@@ -4290,7 +4290,7 @@
       </c>
       <c r="E15" s="14" t="inlineStr">
         <is>
-          <t>技術 翊庭</t>
+          <t>技術 翊庭 / 睿修</t>
         </is>
       </c>
       <c r="F15" s="14" t="inlineStr">
@@ -4322,7 +4322,7 @@
       </c>
       <c r="E16" s="13" t="inlineStr">
         <is>
-          <t>技術 翊庭</t>
+          <t>技術 翊庭 / 睿修</t>
         </is>
       </c>
       <c r="F16" s="13" t="inlineStr">
@@ -4354,7 +4354,7 @@
       </c>
       <c r="E17" s="14" t="inlineStr">
         <is>
-          <t>技術 翊庭 / 人事 芮郗</t>
+          <t>技術 翊庭 / 睿修 / 人事 芮郗</t>
         </is>
       </c>
       <c r="F17" s="14" t="inlineStr">
@@ -4559,7 +4559,7 @@
       </c>
       <c r="F25" s="14" t="inlineStr">
         <is>
-          <t>技術 翊庭 / 人事 芮郗</t>
+          <t>技術 翊庭 / 睿修 / 人事 芮郗</t>
         </is>
       </c>
     </row>
@@ -4623,7 +4623,7 @@
       </c>
       <c r="F27" s="14" t="inlineStr">
         <is>
-          <t>技術 翊庭</t>
+          <t>技術 翊庭 / 睿修</t>
         </is>
       </c>
     </row>
@@ -4818,7 +4818,7 @@
       </c>
       <c r="F6" s="13" t="inlineStr">
         <is>
-          <t>技術 翊庭 / 部門主管</t>
+          <t>技術 翊庭 / 睿修 / 部門主管</t>
         </is>
       </c>
     </row>
@@ -4882,7 +4882,7 @@
       </c>
       <c r="F8" s="13" t="inlineStr">
         <is>
-          <t>技術 翊庭 / 總務 芮郗</t>
+          <t>技術 翊庭 / 睿修 / 總務 芮郗</t>
         </is>
       </c>
     </row>
@@ -5087,7 +5087,7 @@
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>財務 玉霜 / 技術 翊庭 / 人事 芮郗 正式就位，建立文管審查機制</t>
+          <t>財務 玉霜 / 技術 翊庭 / 睿修 / 人事 芮郗 正式就位，建立文管審查機制</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">

</xml_diff>